<commit_message>
add investbook report tip to excel file
</commit_message>
<xml_diff>
--- a/src/main/resources/static/investbook-format-example.xlsx
+++ b/src/main/resources/static/investbook-format-example.xlsx
@@ -15,7 +15,7 @@
     <sheet name="investbook-format-example" sheetId="1" r:id="rId1"/>
     <sheet name="Список допустимых событий" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="152511" refMode="R1C1"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -24,6 +24,40 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Vitek</author>
+  </authors>
+  <commentList>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Vitek:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Обязательно для облигаций, даже если равен 0</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="41">
   <si>
@@ -163,7 +197,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy\ h:mm:ss"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -180,6 +214,19 @@
       <family val="2"/>
       <charset val="204"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -506,7 +553,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K24"/>
   <sheetFormatPr defaultColWidth="15.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1075,6 +1122,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">

</xml_diff>